<commit_message>
chore(license): add nist oscal license file
</commit_message>
<xml_diff>
--- a/project/excel/nist_sp_800_171.xlsx
+++ b/project/excel/nist_sp_800_171.xlsx
@@ -22,10 +22,11 @@
     <sheet name="ControlGroup" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="Control" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="Parameter" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Guideline" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Property" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Link" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Part" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="ParameterSelection" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Guideline" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Property" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Link" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Part" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -677,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -693,35 +694,40 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>select</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>title</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>_class</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>props</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>links</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>parts</t>
         </is>
@@ -729,7 +735,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"family,requirement"</formula1>
     </dataValidation>
   </dataValidations>
@@ -743,6 +749,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>how-many</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>choice</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"one,one-or-more"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -758,7 +795,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -794,7 +831,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -820,7 +857,43 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>metadata</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>groups</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>back-matter</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -876,7 +949,145 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>last-modified</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>version</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>oscal-version</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>props</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>links</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>roles</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>parties</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>responsible-parties</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>short-name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>email-addresses</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>addresses</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -888,283 +1099,109 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>addr-lines</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>postal-code</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>role-id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>party-uuids</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>resources</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>uuid</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>metadata</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>groups</t>
+          <t>description</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>back-matter</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>published</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>last-modified</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>version</t>
+          <t>citation</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>oscal-version</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>props</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>links</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>roles</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>parties</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>responsible-parties</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>type</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>short-name</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>email-addresses</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>addresses</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>addr-lines</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>city</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>state</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>postal-code</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>role-id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>party-uuids</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>resources</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>citation</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
           <t>rlinks</t>
         </is>
       </c>

</xml_diff>